<commit_message>
Initialisation of stocks with  sector + country and etf / stock from admin completed
</commit_message>
<xml_diff>
--- a/src/asset/excel/official_stocks_api.xlsx
+++ b/src/asset/excel/official_stocks_api.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexi\Desktop\ESGICours\pa_5_anne\code\WalletAnalyser-Backend\src\asset\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DE191AE-B5B7-40F3-951C-559B344CB2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B724DE9-AFAA-4501-99B0-883E68A9CF48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="9090" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="9090" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="usa_fr" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18000" uniqueCount="4145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18000" uniqueCount="4147">
   <si>
     <t>NVDA</t>
   </si>
@@ -12465,6 +12465,12 @@
   </si>
   <si>
     <t>États-Unis</t>
+  </si>
+  <si>
+    <t>TOT</t>
+  </si>
+  <si>
+    <t>HSBC</t>
   </si>
 </sst>
 </file>
@@ -40022,7 +40028,7 @@
         <v>1075</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>1082</v>
+        <v>4145</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.75">
@@ -76743,7 +76749,7 @@
         <v>2597</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1047</v>
+        <v>4146</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.75">
@@ -76813,7 +76819,7 @@
         <v>1075</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>1082</v>
+        <v>4145</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.75">

</xml_diff>